<commit_message>
Update annexes with Spearman and Shannon/observed results
Annexes 6 and 7 now report only Spearman correlation and include the
comparison figures. Annexes 10 and 13 use Shannon and observed richness
only; annex 10 is recomputed with crop rotation assigned by SRR ID.
Flatten nested folders and drop scripts copied into annex 11.
</commit_message>
<xml_diff>
--- a/Anexo_10_Diversidad_PRJNA1020132/Anexo_10_Diversidad_PRJNA1020132.xlsx
+++ b/Anexo_10_Diversidad_PRJNA1020132/Anexo_10_Diversidad_PRJNA1020132.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:D89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,15 +431,10 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Simpson</t>
+          <t>Observados</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
-        <is>
-          <t>Chao1</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
@@ -455,12 +450,9 @@
         <v>4.727913615323832</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9818233613955352</v>
-      </c>
-      <c r="D2" t="n">
         <v>233</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -476,12 +468,9 @@
         <v>4.37342753930256</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9595839837589004</v>
-      </c>
-      <c r="D3" t="n">
         <v>203</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -497,14 +486,11 @@
         <v>4.268113636013911</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9621993449367908</v>
-      </c>
-      <c r="D4" t="n">
         <v>158</v>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -518,14 +504,11 @@
         <v>4.019301000420485</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9585912556041788</v>
-      </c>
-      <c r="D5" t="n">
         <v>112</v>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -539,14 +522,11 @@
         <v>4.680088140459228</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9723289162052944</v>
-      </c>
-      <c r="D6" t="n">
         <v>260</v>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -560,12 +540,9 @@
         <v>4.643242956666275</v>
       </c>
       <c r="C7" t="n">
-        <v>0.9743035026411844</v>
-      </c>
-      <c r="D7" t="n">
         <v>219</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -581,12 +558,9 @@
         <v>4.515375378087538</v>
       </c>
       <c r="C8" t="n">
-        <v>0.9690128980909134</v>
-      </c>
-      <c r="D8" t="n">
         <v>217</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -602,14 +576,11 @@
         <v>4.601787336159488</v>
       </c>
       <c r="C9" t="n">
-        <v>0.9682982797847656</v>
-      </c>
-      <c r="D9" t="n">
         <v>252</v>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -623,14 +594,11 @@
         <v>4.675305389147026</v>
       </c>
       <c r="C10" t="n">
-        <v>0.9705240292591616</v>
-      </c>
-      <c r="D10" t="n">
         <v>266</v>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -644,12 +612,9 @@
         <v>4.436698877796648</v>
       </c>
       <c r="C11" t="n">
-        <v>0.9646834284169216</v>
-      </c>
-      <c r="D11" t="n">
         <v>224</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -665,12 +630,9 @@
         <v>4.987932758016299</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9864593000436572</v>
-      </c>
-      <c r="D12" t="n">
         <v>270</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -686,14 +648,11 @@
         <v>4.401628644301807</v>
       </c>
       <c r="C13" t="n">
-        <v>0.9661495561074924</v>
-      </c>
-      <c r="D13" t="n">
         <v>180</v>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -707,14 +666,11 @@
         <v>4.747930759871308</v>
       </c>
       <c r="C14" t="n">
-        <v>0.984348063851576</v>
-      </c>
-      <c r="D14" t="n">
         <v>189</v>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -728,14 +684,11 @@
         <v>4.785548839520375</v>
       </c>
       <c r="C15" t="n">
-        <v>0.9815275535976083</v>
-      </c>
-      <c r="D15" t="n">
         <v>220</v>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -749,12 +702,9 @@
         <v>4.969144551216438</v>
       </c>
       <c r="C16" t="n">
-        <v>0.9880342781366822</v>
-      </c>
-      <c r="D16" t="n">
         <v>234</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -770,12 +720,9 @@
         <v>4.964239510317395</v>
       </c>
       <c r="C17" t="n">
-        <v>0.9876436016364278</v>
-      </c>
-      <c r="D17" t="n">
         <v>240</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -791,14 +738,11 @@
         <v>5.139509278002505</v>
       </c>
       <c r="C18" t="n">
-        <v>0.9905810493401536</v>
-      </c>
-      <c r="D18" t="n">
         <v>277</v>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -812,14 +756,11 @@
         <v>5.025267768569615</v>
       </c>
       <c r="C19" t="n">
-        <v>0.988903600356925</v>
-      </c>
-      <c r="D19" t="n">
         <v>258</v>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -833,12 +774,9 @@
         <v>4.840966567376717</v>
       </c>
       <c r="C20" t="n">
-        <v>0.9842628132387724</v>
-      </c>
-      <c r="D20" t="n">
         <v>239</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -854,12 +792,9 @@
         <v>4.700801148148279</v>
       </c>
       <c r="C21" t="n">
-        <v>0.9693781710888032</v>
-      </c>
-      <c r="D21" t="n">
         <v>283</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -875,14 +810,11 @@
         <v>4.057676006429582</v>
       </c>
       <c r="C22" t="n">
-        <v>0.9545139318813272</v>
-      </c>
-      <c r="D22" t="n">
         <v>131</v>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -896,14 +828,11 @@
         <v>4.400390430211783</v>
       </c>
       <c r="C23" t="n">
-        <v>0.9678631799175732</v>
-      </c>
-      <c r="D23" t="n">
         <v>179</v>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -917,12 +846,9 @@
         <v>4.415815763338032</v>
       </c>
       <c r="C24" t="n">
-        <v>0.9650582261752388</v>
-      </c>
-      <c r="D24" t="n">
         <v>201</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -938,14 +864,11 @@
         <v>4.853747606986211</v>
       </c>
       <c r="C25" t="n">
-        <v>0.9780574505045432</v>
-      </c>
-      <c r="D25" t="n">
         <v>289</v>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -959,14 +882,11 @@
         <v>4.355451529426168</v>
       </c>
       <c r="C26" t="n">
-        <v>0.9658314914311978</v>
-      </c>
-      <c r="D26" t="n">
         <v>179</v>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -980,12 +900,9 @@
         <v>4.163731175537002</v>
       </c>
       <c r="C27" t="n">
-        <v>0.9613969871002348</v>
-      </c>
-      <c r="D27" t="n">
         <v>134</v>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -1001,14 +918,11 @@
         <v>4.811730729087116</v>
       </c>
       <c r="C28" t="n">
-        <v>0.9845922673592008</v>
-      </c>
-      <c r="D28" t="n">
         <v>223</v>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -1022,14 +936,11 @@
         <v>4.430842808299833</v>
       </c>
       <c r="C29" t="n">
-        <v>0.9663694285795896</v>
-      </c>
-      <c r="D29" t="n">
         <v>198</v>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -1043,12 +954,9 @@
         <v>4.87415521476794</v>
       </c>
       <c r="C30" t="n">
-        <v>0.9846016181050332</v>
-      </c>
-      <c r="D30" t="n">
         <v>248</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -1064,12 +972,9 @@
         <v>4.881550062673192</v>
       </c>
       <c r="C31" t="n">
-        <v>0.985401710192078</v>
-      </c>
-      <c r="D31" t="n">
         <v>242</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -1085,12 +990,9 @@
         <v>4.284590212347853</v>
       </c>
       <c r="C32" t="n">
-        <v>0.9712230364493182</v>
-      </c>
-      <c r="D32" t="n">
         <v>153</v>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -1106,12 +1008,9 @@
         <v>4.540152916504041</v>
       </c>
       <c r="C33" t="n">
-        <v>0.9708091126355658</v>
-      </c>
-      <c r="D33" t="n">
         <v>246</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -1127,14 +1026,11 @@
         <v>3.799112558475625</v>
       </c>
       <c r="C34" t="n">
-        <v>0.94621143489754</v>
-      </c>
-      <c r="D34" t="n">
         <v>98</v>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -1148,12 +1044,9 @@
         <v>4.329158971727574</v>
       </c>
       <c r="C35" t="n">
-        <v>0.9663743991563868</v>
-      </c>
-      <c r="D35" t="n">
         <v>158</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -1169,12 +1062,9 @@
         <v>4.42576867445196</v>
       </c>
       <c r="C36" t="n">
-        <v>0.9652718932704882</v>
-      </c>
-      <c r="D36" t="n">
         <v>201</v>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -1190,12 +1080,9 @@
         <v>4.61782104673466</v>
       </c>
       <c r="C37" t="n">
-        <v>0.9696772147084194</v>
-      </c>
-      <c r="D37" t="n">
         <v>257</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -1211,14 +1098,11 @@
         <v>4.254498613836764</v>
       </c>
       <c r="C38" t="n">
-        <v>0.9648291308071676</v>
-      </c>
-      <c r="D38" t="n">
         <v>152</v>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -1232,12 +1116,9 @@
         <v>4.499986607347755</v>
       </c>
       <c r="C39" t="n">
-        <v>0.9675662547703084</v>
-      </c>
-      <c r="D39" t="n">
         <v>216</v>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -1253,14 +1134,11 @@
         <v>3.954052229406671</v>
       </c>
       <c r="C40" t="n">
-        <v>0.9526314537005802</v>
-      </c>
-      <c r="D40" t="n">
         <v>112</v>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -1274,14 +1152,11 @@
         <v>4.792466432912013</v>
       </c>
       <c r="C41" t="n">
-        <v>0.97874392094326</v>
-      </c>
-      <c r="D41" t="n">
         <v>279</v>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -1295,12 +1170,9 @@
         <v>4.291921695864335</v>
       </c>
       <c r="C42" t="n">
-        <v>0.968457696359822</v>
-      </c>
-      <c r="D42" t="n">
         <v>143</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -1316,14 +1188,11 @@
         <v>4.887899818905326</v>
       </c>
       <c r="C43" t="n">
-        <v>0.977240807168744</v>
-      </c>
-      <c r="D43" t="n">
         <v>319</v>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -1337,14 +1206,11 @@
         <v>4.491517207814678</v>
       </c>
       <c r="C44" t="n">
-        <v>0.9689940517355712</v>
-      </c>
-      <c r="D44" t="n">
         <v>196</v>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -1358,14 +1224,11 @@
         <v>4.213295785027315</v>
       </c>
       <c r="C45" t="n">
-        <v>0.9730485804853222</v>
-      </c>
-      <c r="D45" t="n">
         <v>122</v>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1242,9 @@
         <v>4.430286506957092</v>
       </c>
       <c r="C46" t="n">
-        <v>0.9714940992998384</v>
-      </c>
-      <c r="D46" t="n">
         <v>235</v>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -1400,12 +1260,9 @@
         <v>4.639149529513643</v>
       </c>
       <c r="C47" t="n">
-        <v>0.9699051698065956</v>
-      </c>
-      <c r="D47" t="n">
         <v>269</v>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -1421,14 +1278,11 @@
         <v>4.536588828758447</v>
       </c>
       <c r="C48" t="n">
-        <v>0.9671712105552724</v>
-      </c>
-      <c r="D48" t="n">
         <v>225</v>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -1442,14 +1296,11 @@
         <v>4.32887023563142</v>
       </c>
       <c r="C49" t="n">
-        <v>0.9622626114595932</v>
-      </c>
-      <c r="D49" t="n">
         <v>186</v>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -1463,12 +1314,9 @@
         <v>4.373133333980642</v>
       </c>
       <c r="C50" t="n">
-        <v>0.960295603886676</v>
-      </c>
-      <c r="D50" t="n">
         <v>217</v>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -1484,12 +1332,9 @@
         <v>5.008456459697701</v>
       </c>
       <c r="C51" t="n">
-        <v>0.9872026593528956</v>
-      </c>
-      <c r="D51" t="n">
         <v>273</v>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -1505,14 +1350,11 @@
         <v>4.851250460746227</v>
       </c>
       <c r="C52" t="n">
-        <v>0.987522573569022</v>
-      </c>
-      <c r="D52" t="n">
         <v>191</v>
       </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -1526,14 +1368,11 @@
         <v>4.448409326496159</v>
       </c>
       <c r="C53" t="n">
-        <v>0.9804160758686452</v>
-      </c>
-      <c r="D53" t="n">
         <v>134</v>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -1547,14 +1386,11 @@
         <v>4.590282721588087</v>
       </c>
       <c r="C54" t="n">
-        <v>0.9722686823557062</v>
-      </c>
-      <c r="D54" t="n">
         <v>217</v>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -1568,12 +1404,9 @@
         <v>4.808761220034736</v>
       </c>
       <c r="C55" t="n">
-        <v>0.9837778070504468</v>
-      </c>
-      <c r="D55" t="n">
         <v>203</v>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -1589,12 +1422,9 @@
         <v>4.519958174258856</v>
       </c>
       <c r="C56" t="n">
-        <v>0.9761185393593248</v>
-      </c>
-      <c r="D56" t="n">
         <v>185</v>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -1610,14 +1440,11 @@
         <v>4.7948339494373</v>
       </c>
       <c r="C57" t="n">
-        <v>0.9864890724676432</v>
-      </c>
-      <c r="D57" t="n">
         <v>185</v>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -1631,14 +1458,11 @@
         <v>4.936613990224418</v>
       </c>
       <c r="C58" t="n">
-        <v>0.9892082232339195</v>
-      </c>
-      <c r="D58" t="n">
         <v>203</v>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -1652,12 +1476,9 @@
         <v>4.964219265592137</v>
       </c>
       <c r="C59" t="n">
-        <v>0.988269478480832</v>
-      </c>
-      <c r="D59" t="n">
         <v>231</v>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -1673,12 +1494,9 @@
         <v>4.27416907269034</v>
       </c>
       <c r="C60" t="n">
-        <v>0.9608808168591484</v>
-      </c>
-      <c r="D60" t="n">
         <v>166</v>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="D60" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -1694,14 +1512,11 @@
         <v>4.213304207885006</v>
       </c>
       <c r="C61" t="n">
-        <v>0.9600681362131128</v>
-      </c>
-      <c r="D61" t="n">
         <v>153</v>
       </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -1715,14 +1530,11 @@
         <v>4.354497495741709</v>
       </c>
       <c r="C62" t="n">
-        <v>0.9643847826480852</v>
-      </c>
-      <c r="D62" t="n">
         <v>168</v>
       </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1548,9 @@
         <v>4.631200953805885</v>
       </c>
       <c r="C63" t="n">
-        <v>0.9730415519237086</v>
-      </c>
-      <c r="D63" t="n">
         <v>219</v>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -1757,12 +1566,9 @@
         <v>4.241500386030912</v>
       </c>
       <c r="C64" t="n">
-        <v>0.9665287776847586</v>
-      </c>
-      <c r="D64" t="n">
         <v>137</v>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -1778,12 +1584,9 @@
         <v>4.122958924626568</v>
       </c>
       <c r="C65" t="n">
-        <v>0.9663188839167064</v>
-      </c>
-      <c r="D65" t="n">
         <v>113</v>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="D65" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
@@ -1799,14 +1602,11 @@
         <v>4.428978985527641</v>
       </c>
       <c r="C66" t="n">
-        <v>0.9664863259579231</v>
-      </c>
-      <c r="D66" t="n">
         <v>193</v>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -1820,14 +1620,11 @@
         <v>4.45235964743468</v>
       </c>
       <c r="C67" t="n">
-        <v>0.9671459419568974</v>
-      </c>
-      <c r="D67" t="n">
         <v>192</v>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>CS</t>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -1841,14 +1638,11 @@
         <v>4.018109432643039</v>
       </c>
       <c r="C68" t="n">
-        <v>0.9586700472047608</v>
-      </c>
-      <c r="D68" t="n">
         <v>108</v>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -1862,14 +1656,11 @@
         <v>4.850724154771048</v>
       </c>
       <c r="C69" t="n">
-        <v>0.9849157457414252</v>
-      </c>
-      <c r="D69" t="n">
         <v>223</v>
       </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -1883,12 +1674,9 @@
         <v>5.18004509987883</v>
       </c>
       <c r="C70" t="n">
-        <v>0.9900539626060938</v>
-      </c>
-      <c r="D70" t="n">
         <v>295</v>
       </c>
-      <c r="E70" t="inlineStr">
+      <c r="D70" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -1904,12 +1692,9 @@
         <v>5.177522108733596</v>
       </c>
       <c r="C71" t="n">
-        <v>0.9893964430535704</v>
-      </c>
-      <c r="D71" t="n">
         <v>308</v>
       </c>
-      <c r="E71" t="inlineStr">
+      <c r="D71" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -1925,14 +1710,11 @@
         <v>4.819807792710856</v>
       </c>
       <c r="C72" t="n">
-        <v>0.9872906755382244</v>
-      </c>
-      <c r="D72" t="n">
         <v>183</v>
       </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -1946,14 +1728,11 @@
         <v>5.033483219688343</v>
       </c>
       <c r="C73" t="n">
-        <v>0.987677538470097</v>
-      </c>
-      <c r="D73" t="n">
         <v>260</v>
       </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -1967,12 +1746,9 @@
         <v>4.997528953831365</v>
       </c>
       <c r="C74" t="n">
-        <v>0.9900450164124014</v>
-      </c>
-      <c r="D74" t="n">
         <v>212</v>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -1988,12 +1764,9 @@
         <v>4.755990553387885</v>
       </c>
       <c r="C75" t="n">
-        <v>0.986165974832938</v>
-      </c>
-      <c r="D75" t="n">
         <v>174</v>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -2009,14 +1782,11 @@
         <v>3.835042688837456</v>
       </c>
       <c r="C76" t="n">
-        <v>0.9572542943723286</v>
-      </c>
-      <c r="D76" t="n">
         <v>83</v>
       </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -2030,14 +1800,11 @@
         <v>5.122212643389764</v>
       </c>
       <c r="C77" t="n">
-        <v>0.98836216949314</v>
-      </c>
-      <c r="D77" t="n">
         <v>320</v>
       </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -2051,14 +1818,11 @@
         <v>4.451409707690437</v>
       </c>
       <c r="C78" t="n">
-        <v>0.9615006453220528</v>
-      </c>
-      <c r="D78" t="n">
         <v>230</v>
       </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -2072,12 +1836,9 @@
         <v>4.913172138488332</v>
       </c>
       <c r="C79" t="n">
-        <v>0.9839721768068892</v>
-      </c>
-      <c r="D79" t="n">
         <v>272</v>
       </c>
-      <c r="E79" t="inlineStr">
+      <c r="D79" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -2093,12 +1854,9 @@
         <v>4.707035337689703</v>
       </c>
       <c r="C80" t="n">
-        <v>0.979318553428944</v>
-      </c>
-      <c r="D80" t="n">
         <v>222</v>
       </c>
-      <c r="E80" t="inlineStr">
+      <c r="D80" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -2114,14 +1872,11 @@
         <v>4.600365112815678</v>
       </c>
       <c r="C81" t="n">
-        <v>0.982083390579621</v>
-      </c>
-      <c r="D81" t="n">
         <v>172</v>
       </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -2135,12 +1890,9 @@
         <v>4.483702741359124</v>
       </c>
       <c r="C82" t="n">
-        <v>0.9691782154917524</v>
-      </c>
-      <c r="D82" t="n">
         <v>184</v>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="D82" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -2156,12 +1908,9 @@
         <v>4.221860899651439</v>
       </c>
       <c r="C83" t="n">
-        <v>0.9604024402483048</v>
-      </c>
-      <c r="D83" t="n">
         <v>154</v>
       </c>
-      <c r="E83" t="inlineStr">
+      <c r="D83" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -2177,14 +1926,11 @@
         <v>4.203876500464943</v>
       </c>
       <c r="C84" t="n">
-        <v>0.978657603297686</v>
-      </c>
-      <c r="D84" t="n">
         <v>102</v>
       </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Control</t>
         </is>
       </c>
     </row>
@@ -2198,14 +1944,11 @@
         <v>4.075283745806841</v>
       </c>
       <c r="C85" t="n">
-        <v>0.9535762281327984</v>
-      </c>
-      <c r="D85" t="n">
         <v>141</v>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -2219,12 +1962,9 @@
         <v>4.460856250790559</v>
       </c>
       <c r="C86" t="n">
-        <v>0.977926518500195</v>
-      </c>
-      <c r="D86" t="n">
         <v>173</v>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="D86" t="inlineStr">
         <is>
           <t>CSSwP</t>
         </is>
@@ -2240,14 +1980,11 @@
         <v>4.462086775311617</v>
       </c>
       <c r="C87" t="n">
-        <v>0.9761037662412548</v>
-      </c>
-      <c r="D87" t="n">
         <v>189</v>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Sin metadata</t>
         </is>
       </c>
     </row>
@@ -2261,14 +1998,11 @@
         <v>4.004017774919607</v>
       </c>
       <c r="C88" t="n">
-        <v>0.9570559004673568</v>
-      </c>
-      <c r="D88" t="n">
         <v>151</v>
       </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -2282,14 +2016,11 @@
         <v>4.566283715768781</v>
       </c>
       <c r="C89" t="n">
-        <v>0.9637022520347004</v>
-      </c>
-      <c r="D89" t="n">
         <v>270</v>
       </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>CSSwP</t>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2331,36 +2062,23 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1060</v>
+        <v>903</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4451076222831162</v>
+        <v>0.8560717948523305</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Simpson</t>
+          <t>Observados</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1008</v>
+        <v>1001</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7416719182569518</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Chao1</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1072</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.387688654980924</v>
+        <v>0.5115215916067976</v>
       </c>
     </row>
   </sheetData>
@@ -2442,14 +2160,14 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.3556316220333445</v>
+        <v>-0.3556316220333446</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0116826198988604</v>
+        <v>0.01168261989886</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -2463,11 +2181,11 @@
         <v>-0.3666950874251473</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0360504689195918</v>
+        <v>0.0360504689195915</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -2481,11 +2199,11 @@
         <v>-0.3389182162553093</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0012785690026344</v>
+        <v>0.0012785690026345</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2257,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -2557,7 +2275,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2329,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -2625,11 +2343,11 @@
         <v>0.4777117795488325</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.048642469917585</v>
+        <v>-0.0486424699175851</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -2640,14 +2358,14 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.4427576725726543</v>
+        <v>0.4427576725726542</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.0222657017554232</v>
+        <v>-0.0222657017554233</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -2697,11 +2415,11 @@
         <v>0.4415395319018175</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.1097574462742457</v>
+        <v>-0.1097574462742458</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -2719,7 +2437,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -2733,7 +2451,7 @@
         <v>0.4671789981864702</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.0660703758122593</v>
+        <v>-0.0660703758122592</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2773,7 +2491,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2509,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2545,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2563,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -2877,11 +2595,11 @@
         <v>0.510907172899751</v>
       </c>
       <c r="C28" t="n">
-        <v>0.0269048572763981</v>
+        <v>0.0269048572763982</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -2899,7 +2617,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2649,7 @@
         <v>0.5279040109553492</v>
       </c>
       <c r="C31" t="n">
-        <v>0.09245572520330041</v>
+        <v>0.0924557252033005</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2989,7 +2707,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3061,7 +2779,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3097,7 +2815,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3108,14 +2826,14 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.5214751954409831</v>
+        <v>0.5214751954409832</v>
       </c>
       <c r="C41" t="n">
         <v>0.0726001173259738</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3129,7 +2847,7 @@
         <v>-0.3690733252201084</v>
       </c>
       <c r="C42" t="n">
-        <v>0.0264440150339183</v>
+        <v>0.0264440150339182</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -3151,7 +2869,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3169,7 +2887,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3187,7 +2905,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3198,10 +2916,10 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.5209584369697391</v>
+        <v>0.5209584369697392</v>
       </c>
       <c r="C46" t="n">
-        <v>0.3341340705637853</v>
+        <v>0.3341340705637855</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -3219,7 +2937,7 @@
         <v>-0.34808972601082</v>
       </c>
       <c r="C47" t="n">
-        <v>0.007876875096746901</v>
+        <v>0.007876875096746999</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3241,7 +2959,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -3255,11 +2973,11 @@
         <v>-0.3685368792531704</v>
       </c>
       <c r="C49" t="n">
-        <v>0.0167160696419433</v>
+        <v>0.0167160696419432</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -3309,11 +3027,11 @@
         <v>0.3616990651919713</v>
       </c>
       <c r="C52" t="n">
-        <v>-0.1644188583084117</v>
+        <v>-0.1644188583084118</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -3327,11 +3045,11 @@
         <v>0.3826020945880666</v>
       </c>
       <c r="C53" t="n">
-        <v>-0.2002113428306418</v>
+        <v>-0.200211342830642</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -3349,7 +3067,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -3378,7 +3096,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.3497443264740414</v>
+        <v>0.3497443264740413</v>
       </c>
       <c r="C56" t="n">
         <v>-0.2045475082327115</v>
@@ -3403,7 +3121,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -3417,11 +3135,11 @@
         <v>0.3564142082979051</v>
       </c>
       <c r="C58" t="n">
-        <v>-0.1849198127174697</v>
+        <v>-0.1849198127174698</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3153,7 @@
         <v>0.2291071241196891</v>
       </c>
       <c r="C59" t="n">
-        <v>-0.1852767249133001</v>
+        <v>-0.1852767249133</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3475,7 +3193,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -3486,14 +3204,14 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>-0.3585738156047759</v>
+        <v>-0.358573815604776</v>
       </c>
       <c r="C62" t="n">
         <v>0.0066603283857315</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -3507,7 +3225,7 @@
         <v>-0.3416526068191004</v>
       </c>
       <c r="C63" t="n">
-        <v>-0.011030622373359</v>
+        <v>-0.0110306223733589</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3565,7 +3283,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -3583,7 +3301,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -3597,11 +3315,11 @@
         <v>-0.3736054671312626</v>
       </c>
       <c r="C68" t="n">
-        <v>0.0279351430473872</v>
+        <v>0.0279351430473871</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3619,7 +3337,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3630,7 +3348,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>0.35872381829562</v>
+        <v>0.3587238182956199</v>
       </c>
       <c r="C70" t="n">
         <v>-0.1822393227536042</v>
@@ -3651,7 +3369,7 @@
         <v>0.3601314390630981</v>
       </c>
       <c r="C71" t="n">
-        <v>-0.1577002433638206</v>
+        <v>-0.1577002433638207</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3673,7 +3391,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3409,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3463,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3759,11 +3477,11 @@
         <v>0.375820968815208</v>
       </c>
       <c r="C77" t="n">
-        <v>-0.1799824499823777</v>
+        <v>-0.1799824499823776</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3499,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3795,7 +3513,7 @@
         <v>0.5137857081071431</v>
       </c>
       <c r="C79" t="n">
-        <v>0.1026077482150583</v>
+        <v>0.1026077482150584</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3831,11 +3549,11 @@
         <v>0.5255764809134581</v>
       </c>
       <c r="C81" t="n">
-        <v>0.009390525371448299</v>
+        <v>0.0093905253714484</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3885,11 +3603,11 @@
         <v>0.0687644083511052</v>
       </c>
       <c r="C84" t="n">
-        <v>0.2726312085318035</v>
+        <v>0.2726312085318033</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>Control</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3625,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3639,7 @@
         <v>0.4996068617951564</v>
       </c>
       <c r="C86" t="n">
-        <v>0.3478417181300082</v>
+        <v>0.3478417181300083</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3939,11 +3657,11 @@
         <v>0.5135454384737363</v>
       </c>
       <c r="C87" t="n">
-        <v>0.3606380791457187</v>
+        <v>0.3606380791457189</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>Sin metadata</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3679,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3697,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>CSSwP</t>
+          <t>CS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rerun annex 10 with S1A2 assigned to CSSwP
</commit_message>
<xml_diff>
--- a/Anexo_10_Diversidad_PRJNA1020132/Anexo_10_Diversidad_PRJNA1020132.xlsx
+++ b/Anexo_10_Diversidad_PRJNA1020132/Anexo_10_Diversidad_PRJNA1020132.xlsx
@@ -1984,7 +1984,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Sin metadata</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>
@@ -2062,10 +2062,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>903</v>
+        <v>928</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8560717948523305</v>
+        <v>0.8818941220889477</v>
       </c>
     </row>
     <row r="3">
@@ -2075,10 +2075,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1001</v>
+        <v>1029</v>
       </c>
       <c r="C3" t="n">
-        <v>0.5115215916067976</v>
+        <v>0.4836411750614761</v>
       </c>
     </row>
   </sheetData>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Sin metadata</t>
+          <t>CSSwP</t>
         </is>
       </c>
     </row>

</xml_diff>